<commit_message>
Update snippet mapping based on PR feedback
</commit_message>
<xml_diff>
--- a/snippet-extractor-metadata/excel.xlsx
+++ b/snippet-extractor-metadata/excel.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30013"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30030"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC677896-8741-4F3B-A5BD-9CC686A06A02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CDE45DB-35E5-46D9-B88C-593E645AC22A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-270" windowWidth="38640" windowHeight="21120" xr2:uid="{CB5595D7-4492-4192-A1C1-2583BA1957AA}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{CB5595D7-4492-4192-A1C1-2583BA1957AA}"/>
   </bookViews>
   <sheets>
     <sheet name="Snippets" sheetId="2" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2126" uniqueCount="785">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2126" uniqueCount="784">
   <si>
     <t>Class</t>
   </si>
@@ -2353,9 +2353,6 @@
   </si>
   <si>
     <t>setFillProperties</t>
-  </si>
-  <si>
-    <t>transparency</t>
   </si>
   <si>
     <t>clear</t>
@@ -8190,9 +8187,6 @@
       <c r="C299" t="s">
         <v>272</v>
       </c>
-      <c r="D299">
-        <v>1</v>
-      </c>
       <c r="E299" t="s">
         <v>772</v>
       </c>
@@ -8396,13 +8390,13 @@
         <v>267</v>
       </c>
       <c r="C310" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="E310" t="s">
         <v>772</v>
       </c>
       <c r="F310" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
     </row>
     <row r="311" spans="1:6" x14ac:dyDescent="0.25">
@@ -8529,17 +8523,14 @@
       <c r="B317" t="s">
         <v>771</v>
       </c>
-      <c r="C317" t="s">
-        <v>149</v>
-      </c>
-      <c r="D317">
-        <v>1</v>
+      <c r="D317" t="s">
+        <v>711</v>
       </c>
       <c r="E317" t="s">
         <v>772</v>
       </c>
       <c r="F317" t="s">
-        <v>773</v>
+        <v>774</v>
       </c>
     </row>
     <row r="318" spans="1:6" x14ac:dyDescent="0.25">
@@ -8550,13 +8541,16 @@
         <v>771</v>
       </c>
       <c r="C318" t="s">
-        <v>775</v>
+        <v>149</v>
+      </c>
+      <c r="D318">
+        <v>1</v>
       </c>
       <c r="E318" t="s">
         <v>772</v>
       </c>
       <c r="F318" t="s">
-        <v>774</v>
+        <v>773</v>
       </c>
     </row>
     <row r="319" spans="1:6" x14ac:dyDescent="0.25">
@@ -8567,7 +8561,7 @@
         <v>771</v>
       </c>
       <c r="C319" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="D319">
         <v>1</v>
@@ -8576,7 +8570,7 @@
         <v>772</v>
       </c>
       <c r="F319" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
     </row>
     <row r="320" spans="1:6" x14ac:dyDescent="0.25">
@@ -8604,7 +8598,7 @@
         <v>683</v>
       </c>
       <c r="B321" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
       <c r="C321" t="s">
         <v>30</v>
@@ -8616,7 +8610,7 @@
         <v>772</v>
       </c>
       <c r="F321" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
     </row>
     <row r="322" spans="1:6" x14ac:dyDescent="0.25">
@@ -8624,7 +8618,7 @@
         <v>683</v>
       </c>
       <c r="B322" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
       <c r="C322" t="s">
         <v>545</v>
@@ -8633,7 +8627,7 @@
         <v>772</v>
       </c>
       <c r="F322" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
     </row>
     <row r="323" spans="1:6" x14ac:dyDescent="0.25">
@@ -8641,7 +8635,7 @@
         <v>683</v>
       </c>
       <c r="B323" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="D323" t="s">
         <v>581</v>
@@ -8650,7 +8644,7 @@
         <v>772</v>
       </c>
       <c r="F323" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
     </row>
     <row r="324" spans="1:6" x14ac:dyDescent="0.25">
@@ -8658,7 +8652,7 @@
         <v>683</v>
       </c>
       <c r="B324" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
       <c r="D324" t="s">
         <v>581</v>
@@ -8667,7 +8661,7 @@
         <v>772</v>
       </c>
       <c r="F324" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
     </row>
     <row r="325" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>